<commit_message>
Capture positivity research path and retire stale artifacts
The workspace adds positivity momentum strategy research, wires the mfbt_pos factor variant into EMP008, and removes older generated RRG/EMP008 research outputs that should no longer be carried as active tracked artifacts.

Constraint: User requested commit, push, and merge from the current workspace state

Confidence: medium

Scope-risk: broad

Directive: Treat the large artifact deletion set as intentional only for this commit; verify before reintroducing generated outputs

Tested: python -m pytest tests/strategies/test_positivity.py tests/scripts/test_run_pos_research.py tests/scripts/test_run_pos_strategy_grid.py tests/scripts/test_run_mfbt_emp008_full.py (86 passed)

Tested: python -m compileall backtesting scripts tests

Not-tested: full python -m pytest timed out after 124s before completion

Co-authored-by: OmX <omx@oh-my-codex.dev>
</commit_message>
<xml_diff>
--- a/etfs/refresh/pdf.xlsx
+++ b/etfs/refresh/pdf.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CHECK\Documents\GitHub\shquants\etfs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CHECK\Documents\GitHub\shquants\etfs\refresh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC37720B-CA2A-4C4D-8638-BF26311E6E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC72174D-00E7-4F8F-9BB3-CBBFDDD4ED60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{C945E703-BC4E-4B33-A17F-92AC91BD6D2B}"/>
   </bookViews>

</xml_diff>